<commit_message>
Test. Increased variance. Increased reactive power.
</commit_message>
<xml_diff>
--- a/data/CS7/Market Data/CS7_market_data.xlsx
+++ b/data/CS7/Market Data/CS7_market_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\thesis-shared-resources-planning-no_esso-degradation\data\CS7\Market Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3764F0C-D9D2-4183-9609-11D460B33DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{080D917E-B370-4C1E-97E4-9D9899348410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21375" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-15195" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Growth Factors" sheetId="1" r:id="rId1"/>
@@ -515,76 +515,76 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>91.75</v>
+        <v>97.25500000000001</v>
       </c>
       <c r="D2" s="1">
-        <v>86.18</v>
+        <v>91.350800000000007</v>
       </c>
       <c r="E2" s="1">
-        <v>82.1</v>
+        <v>87.025999999999996</v>
       </c>
       <c r="F2" s="1">
-        <v>80</v>
+        <v>84.800000000000011</v>
       </c>
       <c r="G2" s="1">
-        <v>79.599999999999994</v>
+        <v>84.376000000000005</v>
       </c>
       <c r="H2" s="1">
-        <v>81.099999999999994</v>
+        <v>85.965999999999994</v>
       </c>
       <c r="I2" s="1">
-        <v>85.91</v>
+        <v>91.064599999999999</v>
       </c>
       <c r="J2" s="1">
-        <v>102.05</v>
+        <v>108.173</v>
       </c>
       <c r="K2" s="1">
-        <v>113.84</v>
+        <v>120.67040000000001</v>
       </c>
       <c r="L2" s="1">
-        <v>110</v>
+        <v>116.60000000000001</v>
       </c>
       <c r="M2" s="1">
-        <v>97.63</v>
+        <v>103.48780000000001</v>
       </c>
       <c r="N2" s="1">
-        <v>86.18</v>
+        <v>91.350800000000007</v>
       </c>
       <c r="O2" s="1">
-        <v>83.89</v>
+        <v>88.923400000000001</v>
       </c>
       <c r="P2" s="1">
-        <v>82.18</v>
+        <v>87.110800000000012</v>
       </c>
       <c r="Q2" s="1">
-        <v>83</v>
+        <v>87.98</v>
       </c>
       <c r="R2" s="1">
-        <v>85</v>
+        <v>90.100000000000009</v>
       </c>
       <c r="S2" s="1">
-        <v>97.63</v>
+        <v>103.48780000000001</v>
       </c>
       <c r="T2" s="1">
-        <v>118.5</v>
+        <v>125.61</v>
       </c>
       <c r="U2" s="1">
-        <v>128.93</v>
+        <v>136.66580000000002</v>
       </c>
       <c r="V2" s="1">
-        <v>132.31</v>
+        <v>140.24860000000001</v>
       </c>
       <c r="W2" s="1">
-        <v>117.93</v>
+        <v>125.00580000000001</v>
       </c>
       <c r="X2" s="1">
-        <v>108.33</v>
+        <v>114.82980000000001</v>
       </c>
       <c r="Y2" s="1">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="Z2" s="1">
-        <v>93.26</v>
+        <v>98.85560000000001</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.3">
@@ -595,76 +595,76 @@
         <v>2</v>
       </c>
       <c r="C3" s="1">
-        <v>88.98</v>
+        <v>97.878000000000014</v>
       </c>
       <c r="D3" s="1">
-        <v>86.45</v>
+        <v>95.095000000000013</v>
       </c>
       <c r="E3" s="1">
-        <v>84.99</v>
+        <v>93.489000000000004</v>
       </c>
       <c r="F3" s="1">
-        <v>83</v>
+        <v>91.300000000000011</v>
       </c>
       <c r="G3" s="1">
-        <v>83.14</v>
+        <v>91.454000000000008</v>
       </c>
       <c r="H3" s="1">
-        <v>85</v>
+        <v>93.500000000000014</v>
       </c>
       <c r="I3" s="1">
-        <v>89</v>
+        <v>97.9</v>
       </c>
       <c r="J3" s="1">
-        <v>100</v>
+        <v>110.00000000000001</v>
       </c>
       <c r="K3" s="1">
-        <v>104.77</v>
+        <v>115.247</v>
       </c>
       <c r="L3" s="1">
-        <v>105</v>
+        <v>115.50000000000001</v>
       </c>
       <c r="M3" s="1">
-        <v>100</v>
+        <v>110.00000000000001</v>
       </c>
       <c r="N3" s="1">
-        <v>94.58</v>
+        <v>104.03800000000001</v>
       </c>
       <c r="O3" s="1">
-        <v>92</v>
+        <v>101.2</v>
       </c>
       <c r="P3" s="1">
-        <v>91.78</v>
+        <v>100.95800000000001</v>
       </c>
       <c r="Q3" s="1">
-        <v>90.1</v>
+        <v>99.11</v>
       </c>
       <c r="R3" s="1">
-        <v>92.01</v>
+        <v>101.21100000000001</v>
       </c>
       <c r="S3" s="1">
-        <v>100.98</v>
+        <v>111.07800000000002</v>
       </c>
       <c r="T3" s="1">
-        <v>107.1</v>
+        <v>117.81</v>
       </c>
       <c r="U3" s="1">
-        <v>126</v>
+        <v>138.60000000000002</v>
       </c>
       <c r="V3" s="1">
-        <v>119.47</v>
+        <v>131.417</v>
       </c>
       <c r="W3" s="1">
-        <v>110</v>
+        <v>121.00000000000001</v>
       </c>
       <c r="X3" s="1">
-        <v>102.26</v>
+        <v>112.48600000000002</v>
       </c>
       <c r="Y3" s="1">
-        <v>98</v>
+        <v>107.80000000000001</v>
       </c>
       <c r="Z3" s="1">
-        <v>95.49</v>
+        <v>105.039</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.3">
@@ -675,76 +675,76 @@
         <v>3</v>
       </c>
       <c r="C4" s="1">
-        <v>92.33</v>
+        <v>100.6397</v>
       </c>
       <c r="D4" s="1">
-        <v>90.12</v>
+        <v>98.230800000000016</v>
       </c>
       <c r="E4" s="1">
-        <v>87.01</v>
+        <v>94.840900000000019</v>
       </c>
       <c r="F4" s="1">
-        <v>85.8</v>
+        <v>93.522000000000006</v>
       </c>
       <c r="G4" s="1">
-        <v>85</v>
+        <v>92.65</v>
       </c>
       <c r="H4" s="1">
-        <v>86.3</v>
+        <v>94.067000000000007</v>
       </c>
       <c r="I4" s="1">
-        <v>95</v>
+        <v>103.55000000000001</v>
       </c>
       <c r="J4" s="1">
-        <v>103.94</v>
+        <v>113.2946</v>
       </c>
       <c r="K4" s="1">
-        <v>121.4</v>
+        <v>132.32600000000002</v>
       </c>
       <c r="L4" s="1">
-        <v>121.4</v>
+        <v>132.32600000000002</v>
       </c>
       <c r="M4" s="1">
-        <v>105.38</v>
+        <v>114.8642</v>
       </c>
       <c r="N4" s="1">
-        <v>102.97</v>
+        <v>112.2373</v>
       </c>
       <c r="O4" s="1">
-        <v>99.99</v>
+        <v>108.98910000000001</v>
       </c>
       <c r="P4" s="1">
-        <v>98.5</v>
+        <v>107.36500000000001</v>
       </c>
       <c r="Q4" s="1">
-        <v>94.76</v>
+        <v>103.28840000000001</v>
       </c>
       <c r="R4" s="1">
-        <v>94.73</v>
+        <v>103.25570000000002</v>
       </c>
       <c r="S4" s="1">
-        <v>99.37</v>
+        <v>108.31330000000001</v>
       </c>
       <c r="T4" s="1">
-        <v>102.7</v>
+        <v>111.94300000000001</v>
       </c>
       <c r="U4" s="1">
-        <v>111.29</v>
+        <v>121.30610000000001</v>
       </c>
       <c r="V4" s="1">
-        <v>121.4</v>
+        <v>132.32600000000002</v>
       </c>
       <c r="W4" s="1">
-        <v>120</v>
+        <v>130.80000000000001</v>
       </c>
       <c r="X4" s="1">
-        <v>107.71</v>
+        <v>117.40390000000001</v>
       </c>
       <c r="Y4" s="1">
-        <v>101.32</v>
+        <v>110.4388</v>
       </c>
       <c r="Z4" s="1">
-        <v>92.68</v>
+        <v>101.02120000000002</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.3">
@@ -1565,76 +1565,76 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>57.62807500000001</v>
+        <v>61.085759500000016</v>
       </c>
       <c r="D2" s="1">
-        <v>55.55</v>
+        <v>58.883000000000003</v>
       </c>
       <c r="E2" s="1">
-        <v>53.603549999999998</v>
+        <v>56.819763000000002</v>
       </c>
       <c r="F2" s="1">
-        <v>56.433562500000001</v>
+        <v>59.819576250000004</v>
       </c>
       <c r="G2" s="1">
-        <v>53.282600000000002</v>
+        <v>56.479556000000002</v>
       </c>
       <c r="H2" s="1">
-        <v>54.786250000000003</v>
+        <v>58.073425000000007</v>
       </c>
       <c r="I2" s="1">
-        <v>60.200399999999988</v>
+        <v>63.812423999999993</v>
       </c>
       <c r="J2" s="1">
-        <v>61.536774999999999</v>
+        <v>65.228981500000003</v>
       </c>
       <c r="K2" s="1">
-        <v>56.202299999999994</v>
+        <v>59.574437999999994</v>
       </c>
       <c r="L2" s="1">
-        <v>51.013837500000001</v>
+        <v>54.074667750000003</v>
       </c>
       <c r="M2" s="1">
-        <v>43.947337500000003</v>
+        <v>46.584177750000009</v>
       </c>
       <c r="N2" s="1">
-        <v>42.340462500000001</v>
+        <v>44.88089025</v>
       </c>
       <c r="O2" s="1">
-        <v>36.816000000000003</v>
+        <v>39.024960000000007</v>
       </c>
       <c r="P2" s="1">
-        <v>36.565650000000012</v>
+        <v>38.759589000000013</v>
       </c>
       <c r="Q2" s="1">
-        <v>34.282850000000003</v>
+        <v>36.339821000000008</v>
       </c>
       <c r="R2" s="1">
-        <v>34.995800000000003</v>
+        <v>37.095548000000008</v>
       </c>
       <c r="S2" s="1">
-        <v>41.176437499999999</v>
+        <v>43.647023750000002</v>
       </c>
       <c r="T2" s="1">
-        <v>48.501249999999999</v>
+        <v>51.411324999999998</v>
       </c>
       <c r="U2" s="1">
-        <v>59.501250000000006</v>
+        <v>63.071325000000009</v>
       </c>
       <c r="V2" s="1">
-        <v>65.750237499999997</v>
+        <v>69.695251749999997</v>
       </c>
       <c r="W2" s="1">
-        <v>72.171750000000003</v>
+        <v>76.502055000000013</v>
       </c>
       <c r="X2" s="1">
-        <v>60.631374999999998</v>
+        <v>64.269257499999995</v>
       </c>
       <c r="Y2" s="1">
-        <v>62.711999999999996</v>
+        <v>66.474720000000005</v>
       </c>
       <c r="Z2" s="1">
-        <v>61.610174999999998</v>
+        <v>65.306785500000004</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.3">
@@ -1645,76 +1645,76 @@
         <v>2</v>
       </c>
       <c r="C3" s="1">
-        <v>55.345775000000003</v>
+        <v>54.792317250000004</v>
       </c>
       <c r="D3" s="1">
-        <v>58.327500000000001</v>
+        <v>57.744225</v>
       </c>
       <c r="E3" s="1">
-        <v>57.432374999999993</v>
+        <v>56.858051249999995</v>
       </c>
       <c r="F3" s="1">
-        <v>53.2087875</v>
+        <v>52.676699624999998</v>
       </c>
       <c r="G3" s="1">
-        <v>53.826300000000003</v>
+        <v>53.288037000000003</v>
       </c>
       <c r="H3" s="1">
-        <v>57.525562499999999</v>
+        <v>56.950306874999995</v>
       </c>
       <c r="I3" s="1">
-        <v>60.200399999999988</v>
+        <v>59.598395999999987</v>
       </c>
       <c r="J3" s="1">
-        <v>62.755324999999992</v>
+        <v>62.127771749999994</v>
       </c>
       <c r="K3" s="1">
-        <v>59.040799999999997</v>
+        <v>58.450391999999994</v>
       </c>
       <c r="L3" s="1">
-        <v>49.498575000000002</v>
+        <v>49.003589250000005</v>
       </c>
       <c r="M3" s="1">
-        <v>45.279075000000006</v>
+        <v>44.826284250000008</v>
       </c>
       <c r="N3" s="1">
-        <v>41.5020375</v>
+        <v>41.087017125000003</v>
       </c>
       <c r="O3" s="1">
-        <v>37.1995</v>
+        <v>36.827505000000002</v>
       </c>
       <c r="P3" s="1">
-        <v>36.196300000000008</v>
+        <v>35.834337000000005</v>
       </c>
       <c r="Q3" s="1">
-        <v>33.583200000000005</v>
+        <v>33.247368000000002</v>
       </c>
       <c r="R3" s="1">
-        <v>36.781300000000002</v>
+        <v>36.413487000000003</v>
       </c>
       <c r="S3" s="1">
-        <v>39.953375000000008</v>
+        <v>39.553841250000005</v>
       </c>
       <c r="T3" s="1">
-        <v>46.076187499999996</v>
+        <v>45.615425624999993</v>
       </c>
       <c r="U3" s="1">
-        <v>57.716212500000005</v>
+        <v>57.139050375000004</v>
       </c>
       <c r="V3" s="1">
-        <v>69.817262499999998</v>
+        <v>69.119089875</v>
       </c>
       <c r="W3" s="1">
-        <v>68.047650000000004</v>
+        <v>67.367173500000007</v>
       </c>
       <c r="X3" s="1">
-        <v>62.546049999999994</v>
+        <v>61.920589499999991</v>
       </c>
       <c r="Y3" s="1">
-        <v>59.696999999999996</v>
+        <v>59.100029999999997</v>
       </c>
       <c r="Z3" s="1">
-        <v>60.365524999999998</v>
+        <v>59.761869749999995</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.3">
@@ -1725,76 +1725,76 @@
         <v>3</v>
       </c>
       <c r="C4" s="1">
-        <v>58.769225000000006</v>
+        <v>62.883070750000009</v>
       </c>
       <c r="D4" s="1">
-        <v>53.327999999999996</v>
+        <v>57.060960000000001</v>
       </c>
       <c r="E4" s="1">
-        <v>56.338424999999987</v>
+        <v>60.282114749999991</v>
       </c>
       <c r="F4" s="1">
-        <v>54.283712499999993</v>
+        <v>58.083572374999996</v>
       </c>
       <c r="G4" s="1">
-        <v>57.088500000000003</v>
+        <v>61.084695000000011</v>
       </c>
       <c r="H4" s="1">
-        <v>55.334112499999989</v>
+        <v>59.207500374999995</v>
       </c>
       <c r="I4" s="1">
-        <v>56.727299999999993</v>
+        <v>60.698210999999993</v>
       </c>
       <c r="J4" s="1">
-        <v>60.318224999999991</v>
+        <v>64.540500749999993</v>
       </c>
       <c r="K4" s="1">
-        <v>56.77</v>
+        <v>60.743900000000004</v>
       </c>
       <c r="L4" s="1">
-        <v>53.034187500000002</v>
+        <v>56.746580625000007</v>
       </c>
       <c r="M4" s="1">
-        <v>45.279075000000006</v>
+        <v>48.448610250000009</v>
       </c>
       <c r="N4" s="1">
-        <v>39.825187499999998</v>
+        <v>42.612950625000003</v>
       </c>
       <c r="O4" s="1">
-        <v>37.1995</v>
+        <v>39.803465000000003</v>
       </c>
       <c r="P4" s="1">
-        <v>36.565650000000012</v>
+        <v>39.125245500000013</v>
       </c>
       <c r="Q4" s="1">
-        <v>33.933025000000001</v>
+        <v>36.308336750000002</v>
       </c>
       <c r="R4" s="1">
-        <v>35.352899999999998</v>
+        <v>37.827603000000003</v>
       </c>
       <c r="S4" s="1">
-        <v>39.953375000000008</v>
+        <v>42.75011125000001</v>
       </c>
       <c r="T4" s="1">
-        <v>47.531224999999992</v>
+        <v>50.858410749999997</v>
       </c>
       <c r="U4" s="1">
-        <v>59.501250000000006</v>
+        <v>63.666337500000012</v>
       </c>
       <c r="V4" s="1">
-        <v>69.817262499999998</v>
+        <v>74.704470874999998</v>
       </c>
       <c r="W4" s="1">
-        <v>66.67295</v>
+        <v>71.340056500000003</v>
       </c>
       <c r="X4" s="1">
-        <v>60.631374999999998</v>
+        <v>64.875571250000007</v>
       </c>
       <c r="Y4" s="1">
-        <v>60.902999999999992</v>
+        <v>65.166209999999992</v>
       </c>
       <c r="Z4" s="1">
-        <v>60.987850000000002</v>
+        <v>65.256999500000006</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.3">

</xml_diff>